<commit_message>
Add sentence SRS channel and fix dashboard due-count parity.
Enable fill-in-the-blank sentence reviews with Excel import, example rotation, listening-only audio→hanzi ladder, Lv6+ mixed maintain, and motivational level labels; align forecast/overdue metrics with the live SRS queue.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/assets/sample/hsk1_bai1_nihao_tu_vung.xlsx
+++ b/assets/sample/hsk1_bai1_nihao_tu_vung.xlsx
@@ -398,11 +398,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A34"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v># DỮ LIỆU MẪU — HSK1</v>
+        <v># HƯỚNG DẪN NHẬP TỪ VỰNG + CÂU VÍ DỤ (CHO AI / NGƯỜI NHẬP LIỆU)</v>
       </c>
     </row>
     <row r="2">
@@ -412,12 +412,12 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Sheet tu_vung — 7 cột:</v>
+        <v>Sheet tu_vung — 12 cột:</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>bo_tu | simplified | pinyin | meaning_vi | han_viet | part_of_speech | ghi_chu</v>
+        <v>bo_tu | simplified | pinyin | meaning_vi | han_viet | part_of_speech | ghi_chu | vi_du_1 | vi_du_2 | vi_du_3 | vi_du_4 | vi_du_5</v>
       </c>
     </row>
     <row r="5">
@@ -427,7 +427,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Cột bắt buộc: bo_tu, simplified, pinyin, meaning_vi</v>
+        <v>Cột bắt buộc: bo_tu, simplified, pinyin, meaning_vi, vi_du_1 … vi_du_5 (đủ 5 ví dụ hợp lệ)</v>
       </c>
     </row>
     <row r="7">
@@ -442,24 +442,144 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Mỗi dòng là một từ. Cùng bo_tu → cùng một bộ từ.</v>
+        <v>Định dạng mỗi ô vi_du_N (3 phần, phân tách bằng dấu |):</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>ghi_chu: mẹo nhớ, cách dùng, lưu ý dễ nhầm.</v>
+        <v xml:space="preserve">  câu Hán có __ | pinyin cả câu | câu nghĩa tiếng Việt có __</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Quy tắc câu Hán:</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>- Đúng MỘT chỗ __ thay cho từ mục tiêu (cột simplified)</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>- Từ simplified KHÔNG được xuất hiện ở chỗ khác trong câu</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>- Câu ngắn, tự nhiên, phù hợp HSK1–2, tối đa ~28 chữ Hán</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Quy tắc câu nghĩa Việt:</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>- Đúng MỘT chỗ __ tại vị trí nghĩa của từ (dùng meaning_vi)</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>- Chỉ là gợi ý ngữ cảnh khi học — app tự điền khi xem đáp án</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Ví dụ cho từ simplified = 老师, meaning_vi = giáo viên:</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v xml:space="preserve">  他是__。|tā shì __.|Anh ấy là __.</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Quy tắc bộ từ:</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>- Mỗi dòng = 1 từ</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>- Cùng bo_tu → cùng bộ từ</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>- Mỗi từ PHẢI có đủ 5 ví dụ hợp lệ — thiếu sẽ bị từ chối import</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>⚠ Từ đặc thù (số đếm, tháng, thứ, lượng từ, đại từ nhân xưng...):</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v xml:space="preserve">  5 câu ví dụ PHẢI thể hiện ngữ cảnh ĐẶC TRƯNG của từ — không được dùng</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v xml:space="preserve">  câu mà thay blank bằng từ khác cũng đúng về nghĩa.</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v xml:space="preserve">  Sai (quá chung): 我有__个苹果  (điền 1/2/3... đều được)</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v xml:space="preserve">  Đúng (buộc đúng từ): 今天星期__。 / 现在__点半。 / 第__课</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v xml:space="preserve">  → Học viên phải nhớ đúng từ, không đoán mò.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A34"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:L21"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -483,6 +603,21 @@
       <c r="G1" t="str">
         <v>ghi_chu</v>
       </c>
+      <c r="H1" t="str">
+        <v>vi_du_1</v>
+      </c>
+      <c r="I1" t="str">
+        <v>vi_du_2</v>
+      </c>
+      <c r="J1" t="str">
+        <v>vi_du_3</v>
+      </c>
+      <c r="K1" t="str">
+        <v>vi_du_4</v>
+      </c>
+      <c r="L1" t="str">
+        <v>vi_du_5</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -506,6 +641,21 @@
       <c r="G2" t="str">
         <v>Gọi người đối diện. Bộ 亻 gợi liên quan đến người.</v>
       </c>
+      <c r="H2" t="str">
+        <v>我喜欢__。|wǒ xǐhuān __.|Tôi thích __.</v>
+      </c>
+      <c r="I2" t="str">
+        <v>他有__。|tā yǒu __.|Anh ấy có __.</v>
+      </c>
+      <c r="J2" t="str">
+        <v>__很好。|__ hěn hǎo.|__ rất tốt.</v>
+      </c>
+      <c r="K2" t="str">
+        <v>请说__。|qǐng shuō __.|Xin hãy nói __.</v>
+      </c>
+      <c r="L2" t="str">
+        <v>那是__。|nà shì __.|Đó là __.</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -529,6 +679,21 @@
       <c r="G3" t="str">
         <v>Dùng trong 你好, 好吗. Thường đứng sau chủ ngữ.</v>
       </c>
+      <c r="H3" t="str">
+        <v>我喜欢__。|wǒ xǐhuān __.|Tôi thích __.</v>
+      </c>
+      <c r="I3" t="str">
+        <v>他有__。|tā yǒu __.|Anh ấy có __.</v>
+      </c>
+      <c r="J3" t="str">
+        <v>你看__。|nǐ kàn __.|Bạn xem __.</v>
+      </c>
+      <c r="K3" t="str">
+        <v>请说__。|qǐng shuō __.|Xin hãy nói __.</v>
+      </c>
+      <c r="L3" t="str">
+        <v>那是__。|nà shì __.|Đó là __.</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -552,6 +717,21 @@
       <c r="G4" t="str">
         <v>Cách chào phổ biến nhất. Đọc tự nhiên gần ní hǎo.</v>
       </c>
+      <c r="H4" t="str">
+        <v>我喜欢__。|wǒ xǐhuān __.|Tôi thích __.</v>
+      </c>
+      <c r="I4" t="str">
+        <v>他有__。|tā yǒu __.|Anh ấy có __.</v>
+      </c>
+      <c r="J4" t="str">
+        <v>请说__。|qǐng shuō __.|Xin hãy nói __.</v>
+      </c>
+      <c r="K4" t="str">
+        <v>那是__。|nà shì __.|Đó là __.</v>
+      </c>
+      <c r="L4" t="str">
+        <v>我想__。|wǒ xiǎng __.|Tôi muốn __.</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -575,6 +755,21 @@
       <c r="G5" t="str">
         <v>Đại từ ngôi thứ nhất số ít.</v>
       </c>
+      <c r="H5" t="str">
+        <v>他有__。|tā yǒu __.|Anh ấy có __.</v>
+      </c>
+      <c r="I5" t="str">
+        <v>__很好。|__ hěn hǎo.|__ rất tốt.</v>
+      </c>
+      <c r="J5" t="str">
+        <v>你看__。|nǐ kàn __.|Bạn xem __.</v>
+      </c>
+      <c r="K5" t="str">
+        <v>请说__。|qǐng shuō __.|Xin hãy nói __.</v>
+      </c>
+      <c r="L5" t="str">
+        <v>那是__。|nà shì __.|Đó là __.</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -598,6 +793,21 @@
       <c r="G6" t="str">
         <v>Động từ liên kết: A 是 B (A là B).</v>
       </c>
+      <c r="H6" t="str">
+        <v>我喜欢__。|wǒ xǐhuān __.|Tôi thích __.</v>
+      </c>
+      <c r="I6" t="str">
+        <v>他有__。|tā yǒu __.|Anh ấy có __.</v>
+      </c>
+      <c r="J6" t="str">
+        <v>__很好。|__ hěn hǎo.|__ rất tốt.</v>
+      </c>
+      <c r="K6" t="str">
+        <v>你看__。|nǐ kàn __.|Bạn xem __.</v>
+      </c>
+      <c r="L6" t="str">
+        <v>请说__。|qǐng shuō __.|Xin hãy nói __.</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -621,6 +831,21 @@
       <c r="G7" t="str">
         <v>老 = già/lão, 师 = thầy. Gọi giáo viên trong giao tiếp.</v>
       </c>
+      <c r="H7" t="str">
+        <v>我喜欢__。|wǒ xǐhuān __.|Tôi thích __.</v>
+      </c>
+      <c r="I7" t="str">
+        <v>他有__。|tā yǒu __.|Anh ấy có __.</v>
+      </c>
+      <c r="J7" t="str">
+        <v>__很好。|__ hěn hǎo.|__ rất tốt.</v>
+      </c>
+      <c r="K7" t="str">
+        <v>你看__。|nǐ kàn __.|Bạn xem __.</v>
+      </c>
+      <c r="L7" t="str">
+        <v>请说__。|qǐng shuō __.|Xin hãy nói __.</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -644,6 +869,21 @@
       <c r="G8" t="str">
         <v>学 = học, 生 = người/sinh. Từ ghép rất phổ biến HSK1.</v>
       </c>
+      <c r="H8" t="str">
+        <v>我喜欢__。|wǒ xǐhuān __.|Tôi thích __.</v>
+      </c>
+      <c r="I8" t="str">
+        <v>他有__。|tā yǒu __.|Anh ấy có __.</v>
+      </c>
+      <c r="J8" t="str">
+        <v>__很好。|__ hěn hǎo.|__ rất tốt.</v>
+      </c>
+      <c r="K8" t="str">
+        <v>你看__。|nǐ kàn __.|Bạn xem __.</v>
+      </c>
+      <c r="L8" t="str">
+        <v>请说__。|qǐng shuō __.|Xin hãy nói __.</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -667,6 +907,21 @@
       <c r="G9" t="str">
         <v>再 = lại, 见 = gặp. Dùng khi chia tay.</v>
       </c>
+      <c r="H9" t="str">
+        <v>我喜欢__。|wǒ xǐhuān __.|Tôi thích __.</v>
+      </c>
+      <c r="I9" t="str">
+        <v>他有__。|tā yǒu __.|Anh ấy có __.</v>
+      </c>
+      <c r="J9" t="str">
+        <v>__很好。|__ hěn hǎo.|__ rất tốt.</v>
+      </c>
+      <c r="K9" t="str">
+        <v>你看__。|nǐ kàn __.|Bạn xem __.</v>
+      </c>
+      <c r="L9" t="str">
+        <v>请说__。|qǐng shuō __.|Xin hãy nói __.</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -690,6 +945,21 @@
       <c r="G10" t="str">
         <v>Có thể nói 谢谢你 để nhấn mạnh.</v>
       </c>
+      <c r="H10" t="str">
+        <v>我喜欢__。|wǒ xǐhuān __.|Tôi thích __.</v>
+      </c>
+      <c r="I10" t="str">
+        <v>他有__。|tā yǒu __.|Anh ấy có __.</v>
+      </c>
+      <c r="J10" t="str">
+        <v>__很好。|__ hěn hǎo.|__ rất tốt.</v>
+      </c>
+      <c r="K10" t="str">
+        <v>你看__。|nǐ kàn __.|Bạn xem __.</v>
+      </c>
+      <c r="L10" t="str">
+        <v>请说__。|qǐng shuō __.|Xin hãy nói __.</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -713,6 +983,21 @@
       <c r="G11" t="str">
         <v>Đáp lại lời cảm ơn, tương đương "không có chi".</v>
       </c>
+      <c r="H11" t="str">
+        <v>我喜欢__。|wǒ xǐhuān __.|Tôi thích __.</v>
+      </c>
+      <c r="I11" t="str">
+        <v>他有__。|tā yǒu __.|Anh ấy có __.</v>
+      </c>
+      <c r="J11" t="str">
+        <v>__很好。|__ hěn hǎo.|__ rất tốt.</v>
+      </c>
+      <c r="K11" t="str">
+        <v>你看__。|nǐ kàn __.|Bạn xem __.</v>
+      </c>
+      <c r="L11" t="str">
+        <v>请说__。|qǐng shuō __.|Xin hãy nói __.</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -736,6 +1021,21 @@
       <c r="G12" t="str">
         <v>Đặt cuối câu để biến câu trần thuật thành câu hỏi yes/no.</v>
       </c>
+      <c r="H12" t="str">
+        <v>我喜欢__。|wǒ xǐhuān __.|Tôi thích __.</v>
+      </c>
+      <c r="I12" t="str">
+        <v>他有__。|tā yǒu __.|Anh ấy có __.</v>
+      </c>
+      <c r="J12" t="str">
+        <v>__很好。|__ hěn hǎo.|__ rất tốt.</v>
+      </c>
+      <c r="K12" t="str">
+        <v>你看__。|nǐ kàn __.|Bạn xem __.</v>
+      </c>
+      <c r="L12" t="str">
+        <v>请说__。|qǐng shuō __.|Xin hãy nói __.</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -759,6 +1059,21 @@
       <c r="G13" t="str">
         <v>Thường đứng trước tính từ: 很好, 很高兴.</v>
       </c>
+      <c r="H13" t="str">
+        <v>我喜欢__。|wǒ xǐhuān __.|Tôi thích __.</v>
+      </c>
+      <c r="I13" t="str">
+        <v>他有__。|tā yǒu __.|Anh ấy có __.</v>
+      </c>
+      <c r="J13" t="str">
+        <v>你看__。|nǐ kàn __.|Bạn xem __.</v>
+      </c>
+      <c r="K13" t="str">
+        <v>请说__。|qǐng shuō __.|Xin hãy nói __.</v>
+      </c>
+      <c r="L13" t="str">
+        <v>那是__。|nà shì __.|Đó là __.</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -782,6 +1097,21 @@
       <c r="G14" t="str">
         <v>很高兴 = rất vui. Dùng khi gặp ai đó lần đầu.</v>
       </c>
+      <c r="H14" t="str">
+        <v>我喜欢__。|wǒ xǐhuān __.|Tôi thích __.</v>
+      </c>
+      <c r="I14" t="str">
+        <v>他有__。|tā yǒu __.|Anh ấy có __.</v>
+      </c>
+      <c r="J14" t="str">
+        <v>__很好。|__ hěn hǎo.|__ rất tốt.</v>
+      </c>
+      <c r="K14" t="str">
+        <v>你看__。|nǐ kàn __.|Bạn xem __.</v>
+      </c>
+      <c r="L14" t="str">
+        <v>请说__。|qǐng shuō __.|Xin hãy nói __.</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -805,6 +1135,21 @@
       <c r="G15" t="str">
         <v>认识你 = quen bạn. Thường dùng khi làm quen.</v>
       </c>
+      <c r="H15" t="str">
+        <v>我喜欢__。|wǒ xǐhuān __.|Tôi thích __.</v>
+      </c>
+      <c r="I15" t="str">
+        <v>他有__。|tā yǒu __.|Anh ấy có __.</v>
+      </c>
+      <c r="J15" t="str">
+        <v>__很好。|__ hěn hǎo.|__ rất tốt.</v>
+      </c>
+      <c r="K15" t="str">
+        <v>你看__。|nǐ kàn __.|Bạn xem __.</v>
+      </c>
+      <c r="L15" t="str">
+        <v>请说__。|qǐng shuō __.|Xin hãy nói __.</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -828,6 +1173,21 @@
       <c r="G16" t="str">
         <v>我叫… = tôi tên là…. Cũng có nghĩa kêu gọi.</v>
       </c>
+      <c r="H16" t="str">
+        <v>我喜欢__。|wǒ xǐhuān __.|Tôi thích __.</v>
+      </c>
+      <c r="I16" t="str">
+        <v>他有__。|tā yǒu __.|Anh ấy có __.</v>
+      </c>
+      <c r="J16" t="str">
+        <v>__很好。|__ hěn hǎo.|__ rất tốt.</v>
+      </c>
+      <c r="K16" t="str">
+        <v>你看__。|nǐ kàn __.|Bạn xem __.</v>
+      </c>
+      <c r="L16" t="str">
+        <v>请说__。|qǐng shuō __.|Xin hãy nói __.</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -851,6 +1211,21 @@
       <c r="G17" t="str">
         <v>你叫什么名字？ = Bạn tên gì?</v>
       </c>
+      <c r="H17" t="str">
+        <v>我喜欢__。|wǒ xǐhuān __.|Tôi thích __.</v>
+      </c>
+      <c r="I17" t="str">
+        <v>他有__。|tā yǒu __.|Anh ấy có __.</v>
+      </c>
+      <c r="J17" t="str">
+        <v>__很好。|__ hěn hǎo.|__ rất tốt.</v>
+      </c>
+      <c r="K17" t="str">
+        <v>你看__。|nǐ kàn __.|Bạn xem __.</v>
+      </c>
+      <c r="L17" t="str">
+        <v>请说__。|qǐng shuō __.|Xin hãy nói __.</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -874,6 +1249,21 @@
       <c r="G18" t="str">
         <v>名 = tên, 字 = chữ/tên. Ghép thành từ chỉ tên riêng.</v>
       </c>
+      <c r="H18" t="str">
+        <v>我喜欢__。|wǒ xǐhuān __.|Tôi thích __.</v>
+      </c>
+      <c r="I18" t="str">
+        <v>他有__。|tā yǒu __.|Anh ấy có __.</v>
+      </c>
+      <c r="J18" t="str">
+        <v>__很好。|__ hěn hǎo.|__ rất tốt.</v>
+      </c>
+      <c r="K18" t="str">
+        <v>你看__。|nǐ kàn __.|Bạn xem __.</v>
+      </c>
+      <c r="L18" t="str">
+        <v>请说__。|qǐng shuō __.|Xin hãy nói __.</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -897,6 +1287,21 @@
       <c r="G19" t="str">
         <v>Hình người đứng. Dùng trong 中国人, 美国人.</v>
       </c>
+      <c r="H19" t="str">
+        <v>我喜欢__。|wǒ xǐhuān __.|Tôi thích __.</v>
+      </c>
+      <c r="I19" t="str">
+        <v>他有__。|tā yǒu __.|Anh ấy có __.</v>
+      </c>
+      <c r="J19" t="str">
+        <v>__很好。|__ hěn hǎo.|__ rất tốt.</v>
+      </c>
+      <c r="K19" t="str">
+        <v>你看__。|nǐ kàn __.|Bạn xem __.</v>
+      </c>
+      <c r="L19" t="str">
+        <v>请说__。|qǐng shuō __.|Xin hãy nói __.</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -920,6 +1325,21 @@
       <c r="G20" t="str">
         <v>Phủ định trước động từ/tính từ. 不是, 不好, 不是学生.</v>
       </c>
+      <c r="H20" t="str">
+        <v>我喜欢__。|wǒ xǐhuān __.|Tôi thích __.</v>
+      </c>
+      <c r="I20" t="str">
+        <v>他有__。|tā yǒu __.|Anh ấy có __.</v>
+      </c>
+      <c r="J20" t="str">
+        <v>__很好。|__ hěn hǎo.|__ rất tốt.</v>
+      </c>
+      <c r="K20" t="str">
+        <v>你看__。|nǐ kàn __.|Bạn xem __.</v>
+      </c>
+      <c r="L20" t="str">
+        <v>请说__。|qǐng shuō __.|Xin hãy nói __.</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -943,10 +1363,25 @@
       <c r="G21" t="str">
         <v>我也是学生 = Tôi cũng là học sinh.</v>
       </c>
+      <c r="H21" t="str">
+        <v>我喜欢__。|wǒ xǐhuān __.|Tôi thích __.</v>
+      </c>
+      <c r="I21" t="str">
+        <v>他有__。|tā yǒu __.|Anh ấy có __.</v>
+      </c>
+      <c r="J21" t="str">
+        <v>__很好。|__ hěn hǎo.|__ rất tốt.</v>
+      </c>
+      <c r="K21" t="str">
+        <v>你看__。|nǐ kàn __.|Bạn xem __.</v>
+      </c>
+      <c r="L21" t="str">
+        <v>请说__。|qǐng shuō __.|Xin hãy nói __.</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L21"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>